<commit_message>
docs: confirm IEEE Strand A search re-run
</commit_message>
<xml_diff>
--- a/lit_search/evidence workbook/PRISMA_search_evidence_log.xlsx
+++ b/lit_search/evidence workbook/PRISMA_search_evidence_log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e9ed69ed71ddea64/Documents/GitHub/autonomous_vehicles_arnaud/lit_search/evidence workbook/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="13_ncr:1_{5B94EA4A-FAE7-4C9D-B11E-1C13D2FF80D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{56EF0EC9-3EE2-49FF-A8A3-78C5D6D363E4}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{5B94EA4A-FAE7-4C9D-B11E-1C13D2FF80D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{324C63AB-CE9C-46B9-856C-05FA3FD4B912}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Search Evidence" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="814" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="814" uniqueCount="190">
   <si>
     <t>Strand</t>
   </si>
@@ -661,6 +661,9 @@
   </si>
   <si>
     <t>Stage 2 screening decisions are held in stage_2_abstract_screening_FINAL_20260927.xlsx, frozen 27 September 2026. This sheet is not the file of record.</t>
+  </si>
+  <si>
+    <t>Basic search: ("connected vehicle*" OR "connected and automated vehicle*" OR "autonomous vehicle*" OR "automated vehicle*" OR "self-driving" OR driverless OR "automated driving" OR V2X OR "vehicle-to-everything" OR "vehicle-to-vehicle" OR "vehicle-to-infrastructure"); Search within results: privacy OR "data protection" OR "data security" OR "data sharing" OR "data collection" OR cybersecurity OR "cyber security" OR surveillance OR hacking OR security; Search within results: ("public perception*" OR "public opinion" OR "public attitude*" OR "user perception*" OR acceptance OR "risk perception" OR "social media" OR reddit OR twitter OR forum* OR discourse OR sentiment). Strings recovered 17 October 2026 from the record of the 20 September 2026 session, as supplied for entry immediately before each recorded count; confirmed by re-run on 17 October 2026: 84,356, 13,610, 452 unfiltered, 410 after the 2015–2025 year filter, 337 after the Conferences and Journals filter; screenshot ieee_strandA_rerun_20261017.png.</t>
   </si>
 </sst>
 </file>
@@ -1366,7 +1369,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="63.75">
+    <row r="11" spans="1:9" ht="204">
       <c r="A11" s="7" t="s">
         <v>14</v>
       </c>
@@ -1376,10 +1379,10 @@
       <c r="C11" s="8">
         <v>46285</v>
       </c>
-      <c r="D11" s="9"/>
-      <c r="E11" s="9" t="s">
-        <v>118</v>
-      </c>
+      <c r="D11" s="9" t="s">
+        <v>189</v>
+      </c>
+      <c r="E11" s="9"/>
       <c r="F11" s="5"/>
       <c r="G11" s="5"/>
       <c r="H11" s="7"/>

</xml_diff>